<commit_message>
fix(catalog): tighten juice auto-review package checks and SKU uniqueness
Require real package cues for approved_new, avoid proposed_sku collisions
with existing TINDA SKUs, and refresh juice collection review artifacts.

Co-authored-by: sharipdaitmirzaev-hue <sharipdaitmirzaev-hue@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/imports/zelenoe-yabloko-juice/review-decisions.xlsx
+++ b/data/imports/zelenoe-yabloko-juice/review-decisions.xlsx
@@ -497,10 +497,10 @@
         <v/>
       </c>
       <c r="L2" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M2" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DOBRYI-1000-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N2">
         <v>1024</v>
@@ -515,16 +515,16 @@
         <v>1</v>
       </c>
       <c r="R2">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S2" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T2" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U2" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="3">
@@ -559,10 +559,10 @@
         <v/>
       </c>
       <c r="L3" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M3" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DOBRYI-1000-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N3">
         <v>1024</v>
@@ -577,16 +577,16 @@
         <v>1</v>
       </c>
       <c r="R3">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S3" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T3" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U3" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="4">
@@ -621,10 +621,10 @@
         <v/>
       </c>
       <c r="L4" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M4" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VIKO-1000-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N4">
         <v>550</v>
@@ -639,16 +639,16 @@
         <v>1</v>
       </c>
       <c r="R4">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S4" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T4" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U4" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="5">
@@ -745,10 +745,10 @@
         <v/>
       </c>
       <c r="L6" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M6" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-J7-850-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N6">
         <v>1024</v>
@@ -763,16 +763,16 @@
         <v>1</v>
       </c>
       <c r="R6">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S6" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T6" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U6" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="7">
@@ -1058,10 +1058,10 @@
         <v/>
       </c>
       <c r="L11" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M11" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VIKO-1000-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N11">
         <v>500</v>
@@ -1076,16 +1076,16 @@
         <v>1</v>
       </c>
       <c r="R11">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S11" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T11" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U11" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="12">
@@ -1120,10 +1120,10 @@
         <v/>
       </c>
       <c r="L12" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M12" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VIKO-1000-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N12">
         <v>550</v>
@@ -1138,16 +1138,16 @@
         <v>1</v>
       </c>
       <c r="R12">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S12" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T12" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U12" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="13">
@@ -1182,10 +1182,10 @@
         <v/>
       </c>
       <c r="L13" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M13" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VIKO-1000-UNK-004. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N13">
         <v>550</v>
@@ -1200,16 +1200,16 @@
         <v>1</v>
       </c>
       <c r="R13">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S13" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T13" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U13" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="14">
@@ -1244,10 +1244,10 @@
         <v/>
       </c>
       <c r="L14" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M14" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SIS-1600-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N14">
         <v>900</v>
@@ -1262,16 +1262,16 @@
         <v>1</v>
       </c>
       <c r="R14">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S14" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T14" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U14" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="15">
@@ -1368,10 +1368,10 @@
         <v/>
       </c>
       <c r="L16" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M16" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VIKO-1000-UNK-005. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N16">
         <v>1024</v>
@@ -1386,16 +1386,16 @@
         <v>1</v>
       </c>
       <c r="R16">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S16" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T16" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U16" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="17">
@@ -1492,10 +1492,10 @@
         <v/>
       </c>
       <c r="L18" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M18" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VIKO-1000-UNK-006. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N18">
         <v>550</v>
@@ -1510,16 +1510,16 @@
         <v>1</v>
       </c>
       <c r="R18">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S18" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T18" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U18" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="19">
@@ -1554,10 +1554,10 @@
         <v/>
       </c>
       <c r="L19" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M19" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VIKO-2000-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N19">
         <v>550</v>
@@ -1572,16 +1572,16 @@
         <v>1</v>
       </c>
       <c r="R19">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S19" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T19" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U19" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="20">
@@ -1681,10 +1681,10 @@
         <v/>
       </c>
       <c r="L21" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M21" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SOCHNAYADOLINA-950-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N21">
         <v>500</v>
@@ -1699,16 +1699,16 @@
         <v>1</v>
       </c>
       <c r="R21">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S21" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T21" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U21" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="22">
@@ -2053,10 +2053,10 @@
         <v/>
       </c>
       <c r="L27" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M27" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DOBRYI-1000-UNK-004. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N27">
         <v>585</v>
@@ -2071,16 +2071,16 @@
         <v>1</v>
       </c>
       <c r="R27">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S27" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T27" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U27" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="28">
@@ -2115,10 +2115,10 @@
         <v/>
       </c>
       <c r="L28" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M28" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SOCHNAYADOLINA-950-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N28">
         <v>500</v>
@@ -2133,16 +2133,16 @@
         <v>1</v>
       </c>
       <c r="R28">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S28" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T28" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U28" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="29">
@@ -2239,10 +2239,10 @@
         <v/>
       </c>
       <c r="L30" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M30" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SIS-1600-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N30">
         <v>1024</v>
@@ -2257,16 +2257,16 @@
         <v>1</v>
       </c>
       <c r="R30">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S30" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T30" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U30" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="31">
@@ -2301,10 +2301,10 @@
         <v/>
       </c>
       <c r="L31" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M31" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-RICH-1000-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N31">
         <v>1254</v>
@@ -2319,16 +2319,16 @@
         <v>1</v>
       </c>
       <c r="R31">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S31" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T31" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U31" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="32">
@@ -2363,10 +2363,10 @@
         <v/>
       </c>
       <c r="L32" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M32" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DOBRYI-2000-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N32">
         <v>1254</v>
@@ -2381,16 +2381,16 @@
         <v>1</v>
       </c>
       <c r="R32">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S32" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T32" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U32" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="33">
@@ -2425,10 +2425,10 @@
         <v/>
       </c>
       <c r="L33" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M33" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VIKO-1000-UNK-007. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N33">
         <v>550</v>
@@ -2443,16 +2443,16 @@
         <v>1</v>
       </c>
       <c r="R33">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S33" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T33" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U33" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="34">
@@ -2549,10 +2549,10 @@
         <v/>
       </c>
       <c r="L35" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M35" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-RICH-1000-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N35">
         <v>1024</v>
@@ -2567,16 +2567,16 @@
         <v>1</v>
       </c>
       <c r="R35">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S35" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T35" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U35" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="36">
@@ -2611,10 +2611,10 @@
         <v/>
       </c>
       <c r="L36" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M36" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SIS-1600-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N36">
         <v>1024</v>
@@ -2629,16 +2629,16 @@
         <v>1</v>
       </c>
       <c r="R36">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S36" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T36" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U36" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="37">
@@ -2797,10 +2797,10 @@
         <v/>
       </c>
       <c r="L39" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M39" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VIKO-2000-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N39">
         <v>550</v>
@@ -2815,16 +2815,16 @@
         <v>1</v>
       </c>
       <c r="R39">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S39" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T39" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U39" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="40">
@@ -2859,10 +2859,10 @@
         <v/>
       </c>
       <c r="L40" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M40" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DOBRYI-1000-UNK-005. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N40">
         <v>1000</v>
@@ -2877,16 +2877,16 @@
         <v>1</v>
       </c>
       <c r="R40">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S40" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T40" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U40" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="41">
@@ -2921,10 +2921,10 @@
         <v/>
       </c>
       <c r="L41" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M41" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SADYPRIDONYA-1000-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N41">
         <v>600</v>
@@ -2939,16 +2939,16 @@
         <v>1</v>
       </c>
       <c r="R41">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S41" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|marked_sugar_free|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|marked_sugar_free|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T41" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U41" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="42">
@@ -3169,10 +3169,10 @@
         <v/>
       </c>
       <c r="L45" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M45" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VIKO-2000-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N45">
         <v>1024</v>
@@ -3187,16 +3187,16 @@
         <v>1</v>
       </c>
       <c r="R45">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S45" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T45" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U45" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="46">
@@ -3290,10 +3290,10 @@
         <v/>
       </c>
       <c r="L47" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M47" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SIS-1600-UNK-004. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N47">
         <v>1024</v>
@@ -3308,16 +3308,16 @@
         <v>1</v>
       </c>
       <c r="R47">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S47" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T47" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U47" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="48">
@@ -3352,10 +3352,10 @@
         <v/>
       </c>
       <c r="L48" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M48" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-RICH-1000-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N48">
         <v>1024</v>
@@ -3370,16 +3370,16 @@
         <v>1</v>
       </c>
       <c r="R48">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S48" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T48" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U48" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="49">
@@ -3414,10 +3414,10 @@
         <v/>
       </c>
       <c r="L49" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M49" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SOCHNAYADOLINA-950-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N49">
         <v>500</v>
@@ -3432,16 +3432,16 @@
         <v>1</v>
       </c>
       <c r="R49">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S49" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T49" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U49" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="50">
@@ -3541,10 +3541,10 @@
         <v/>
       </c>
       <c r="L51" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M51" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SADYPRIDONYA-1000-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N51">
         <v>1024</v>
@@ -3559,16 +3559,16 @@
         <v>1</v>
       </c>
       <c r="R51">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S51" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|marked_sugar_free|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|marked_sugar_free|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T51" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U51" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="52">
@@ -3603,10 +3603,10 @@
         <v/>
       </c>
       <c r="L52" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M52" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SADYPRIDONYA-1000-UNK-004. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N52">
         <v>1400</v>
@@ -3621,16 +3621,16 @@
         <v>1</v>
       </c>
       <c r="R52">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S52" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_mors</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_mors</v>
       </c>
       <c r="T52" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U52" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="53">
@@ -3727,10 +3727,10 @@
         <v/>
       </c>
       <c r="L54" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M54" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-MOI-200-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N54">
         <v>700</v>
@@ -3745,16 +3745,16 @@
         <v>1</v>
       </c>
       <c r="R54">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S54" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T54" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U54" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="55">
@@ -3851,10 +3851,10 @@
         <v/>
       </c>
       <c r="L56" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M56" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-J7-300-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N56">
         <v>1024</v>
@@ -3869,16 +3869,16 @@
         <v>1</v>
       </c>
       <c r="R56">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S56" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T56" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U56" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="57">
@@ -4102,10 +4102,10 @@
         <v/>
       </c>
       <c r="L60" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M60" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-RICH-1000-UNK-004. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N60">
         <v>1024</v>
@@ -4120,16 +4120,16 @@
         <v>1</v>
       </c>
       <c r="R60">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S60" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T60" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U60" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="61">
@@ -4226,10 +4226,10 @@
         <v/>
       </c>
       <c r="L62" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M62" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SIS-1600-UNK-005. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N62">
         <v>700</v>
@@ -4244,16 +4244,16 @@
         <v>1</v>
       </c>
       <c r="R62">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S62" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T62" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U62" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="63">
@@ -4412,10 +4412,10 @@
         <v/>
       </c>
       <c r="L65" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M65" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VIKO-2000-UNK-004. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N65">
         <v>500</v>
@@ -4430,16 +4430,16 @@
         <v>1</v>
       </c>
       <c r="R65">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S65" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T65" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U65" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="66">
@@ -4595,10 +4595,10 @@
         <v/>
       </c>
       <c r="L68" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M68" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-MOI-950-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N68">
         <v>600</v>
@@ -4613,16 +4613,16 @@
         <v>1</v>
       </c>
       <c r="R68">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S68" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T68" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U68" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="69">
@@ -4657,10 +4657,10 @@
         <v/>
       </c>
       <c r="L69" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M69" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VIKO-200-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N69">
         <v>500</v>
@@ -4675,16 +4675,16 @@
         <v>1</v>
       </c>
       <c r="R69">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S69" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T69" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U69" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="70">
@@ -4719,10 +4719,10 @@
         <v/>
       </c>
       <c r="L70" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M70" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VIKO-200-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N70">
         <v>1000</v>
@@ -4737,16 +4737,16 @@
         <v>1</v>
       </c>
       <c r="R70">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S70" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T70" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U70" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="71">
@@ -4781,10 +4781,10 @@
         <v/>
       </c>
       <c r="L71" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M71" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-GUNIB-3000-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N71">
         <v>1024</v>
@@ -4799,16 +4799,16 @@
         <v>1</v>
       </c>
       <c r="R71">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S71" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T71" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U71" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="72">
@@ -4905,10 +4905,10 @@
         <v/>
       </c>
       <c r="L73" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M73" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-J7-970-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N73">
         <v>1024</v>
@@ -4923,16 +4923,16 @@
         <v>1</v>
       </c>
       <c r="R73">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S73" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|has_pulp</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|has_pulp</v>
       </c>
       <c r="T73" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U73" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="74">
@@ -5079,10 +5079,10 @@
         <v/>
       </c>
       <c r="L76" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M76" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SADYPRIDONYA-200-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N76">
         <v>1024</v>
@@ -5097,16 +5097,16 @@
         <v>1</v>
       </c>
       <c r="R76">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S76" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T76" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U76" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="77">
@@ -5141,10 +5141,10 @@
         <v/>
       </c>
       <c r="L77" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M77" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SOCHNAYADOLINA-950-UNK-004. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N77">
         <v>500</v>
@@ -5159,16 +5159,16 @@
         <v>1</v>
       </c>
       <c r="R77">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S77" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T77" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U77" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="78">
@@ -5321,10 +5321,10 @@
         <v/>
       </c>
       <c r="L80" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M80" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SADYPRIDONYA-200-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N80">
         <v>1024</v>
@@ -5339,16 +5339,16 @@
         <v>1</v>
       </c>
       <c r="R80">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S80" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T80" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U80" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="81">
@@ -5383,10 +5383,10 @@
         <v/>
       </c>
       <c r="L81" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M81" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SOCHNAYADOLINA-1930-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N81">
         <v>640</v>
@@ -5401,16 +5401,16 @@
         <v>1</v>
       </c>
       <c r="R81">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S81" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T81" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U81" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="82">
@@ -5445,10 +5445,10 @@
         <v/>
       </c>
       <c r="L82" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M82" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DOBRYI-2000-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N82">
         <v>900</v>
@@ -5463,16 +5463,16 @@
         <v>1</v>
       </c>
       <c r="R82">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S82" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T82" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U82" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="83">
@@ -5507,10 +5507,10 @@
         <v/>
       </c>
       <c r="L83" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M83" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-LYUBIMYI-1930-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N83">
         <v>1000</v>
@@ -5525,16 +5525,16 @@
         <v>1</v>
       </c>
       <c r="R83">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S83" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T83" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U83" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="84">
@@ -5569,10 +5569,10 @@
         <v/>
       </c>
       <c r="L84" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M84" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-J7-970-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N84">
         <v>1024</v>
@@ -5587,16 +5587,16 @@
         <v>1</v>
       </c>
       <c r="R84">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S84" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T84" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U84" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="85">
@@ -5631,10 +5631,10 @@
         <v/>
       </c>
       <c r="L85" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M85" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SADYPRIDONYA-200-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N85">
         <v>1000</v>
@@ -5649,16 +5649,16 @@
         <v>1</v>
       </c>
       <c r="R85">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S85" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T85" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U85" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="86">
@@ -5693,10 +5693,10 @@
         <v/>
       </c>
       <c r="L86" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M86" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SADYPRIDONYA-1000-UNK-005. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N86">
         <v>1024</v>
@@ -5711,16 +5711,16 @@
         <v>1</v>
       </c>
       <c r="R86">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S86" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|marked_sugar_free|category_juice_slug|product_type_juice|has_pulp</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|marked_sugar_free|category_juice_slug|product_type_juice|has_pulp</v>
       </c>
       <c r="T86" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U86" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="87">
@@ -5817,10 +5817,10 @@
         <v/>
       </c>
       <c r="L88" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M88" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VIKO-1000-UNK-009. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N88">
         <v>1000</v>
@@ -5835,16 +5835,16 @@
         <v>1</v>
       </c>
       <c r="R88">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S88" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T88" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U88" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="89">
@@ -5941,10 +5941,10 @@
         <v/>
       </c>
       <c r="L90" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M90" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DOBRYI-2000-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N90">
         <v>1000</v>
@@ -5959,16 +5959,16 @@
         <v>1</v>
       </c>
       <c r="R90">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S90" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T90" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U90" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="91">
@@ -6189,10 +6189,10 @@
         <v/>
       </c>
       <c r="L94" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M94" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-J7-970-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N94">
         <v>1024</v>
@@ -6207,16 +6207,16 @@
         <v>1</v>
       </c>
       <c r="R94">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S94" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|has_pulp</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|has_pulp</v>
       </c>
       <c r="T94" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U94" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="95">
@@ -6313,10 +6313,10 @@
         <v/>
       </c>
       <c r="L96" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M96" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SADYPRIDONYA-1000-UNK-006. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N96">
         <v>1024</v>
@@ -6331,16 +6331,16 @@
         <v>1</v>
       </c>
       <c r="R96">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S96" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|marked_sugar_free|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|marked_sugar_free|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T96" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U96" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="97">
@@ -6375,10 +6375,10 @@
         <v/>
       </c>
       <c r="L97" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M97" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SOCHNAYADOLINA-1930-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N97">
         <v>800</v>
@@ -6393,16 +6393,16 @@
         <v>1</v>
       </c>
       <c r="R97">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S97" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T97" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U97" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="98">
@@ -6499,10 +6499,10 @@
         <v/>
       </c>
       <c r="L99" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M99" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SIS-1600-UNK-006. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N99">
         <v>1024</v>
@@ -6517,16 +6517,16 @@
         <v>1</v>
       </c>
       <c r="R99">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S99" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T99" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U99" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="100">
@@ -6561,10 +6561,10 @@
         <v/>
       </c>
       <c r="L100" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M100" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SIS-1600-UNK-007. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N100">
         <v>1024</v>
@@ -6579,16 +6579,16 @@
         <v>1</v>
       </c>
       <c r="R100">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S100" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T100" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U100" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="101">
@@ -6685,10 +6685,10 @@
         <v/>
       </c>
       <c r="L102" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M102" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SOCHNAYADOLINA-950-UNK-006. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N102">
         <v>600</v>
@@ -6703,16 +6703,16 @@
         <v>1</v>
       </c>
       <c r="R102">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S102" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T102" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U102" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="103">
@@ -6747,10 +6747,10 @@
         <v/>
       </c>
       <c r="L103" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M103" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-J7-970-UNK-004. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N103">
         <v>1024</v>
@@ -6765,16 +6765,16 @@
         <v>1</v>
       </c>
       <c r="R103">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S103" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T103" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U103" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="104">
@@ -6809,10 +6809,10 @@
         <v/>
       </c>
       <c r="L104" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M104" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-J7-970-UNK-005. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N104">
         <v>1024</v>
@@ -6827,16 +6827,16 @@
         <v>1</v>
       </c>
       <c r="R104">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S104" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|has_pulp</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|has_pulp</v>
       </c>
       <c r="T104" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U104" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="105">
@@ -6989,10 +6989,10 @@
         <v/>
       </c>
       <c r="L107" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M107" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SADYPRIDONYA-200-UNK-004. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N107">
         <v>1024</v>
@@ -7007,16 +7007,16 @@
         <v>1</v>
       </c>
       <c r="R107">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S107" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T107" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U107" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="108">
@@ -7175,10 +7175,10 @@
         <v/>
       </c>
       <c r="L110" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M110" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DOBRYI-1000-UNK-009. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N110">
         <v>800</v>
@@ -7193,16 +7193,16 @@
         <v>1</v>
       </c>
       <c r="R110">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S110" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T110" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U110" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="111">
@@ -7237,10 +7237,10 @@
         <v/>
       </c>
       <c r="L111" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M111" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SADYPRIDONYA-1000-UNK-007. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N111">
         <v>1400</v>
@@ -7255,16 +7255,16 @@
         <v>1</v>
       </c>
       <c r="R111">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S111" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_mors</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_mors</v>
       </c>
       <c r="T111" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U111" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="112">
@@ -7485,10 +7485,10 @@
         <v/>
       </c>
       <c r="L115" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M115" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-MOI-950-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N115">
         <v>600</v>
@@ -7503,16 +7503,16 @@
         <v>1</v>
       </c>
       <c r="R115">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S115" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T115" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U115" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="116">
@@ -7547,10 +7547,10 @@
         <v/>
       </c>
       <c r="L116" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M116" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-MOI-1930-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N116">
         <v>650</v>
@@ -7565,16 +7565,16 @@
         <v>1</v>
       </c>
       <c r="R116">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S116" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T116" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U116" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="117">
@@ -7671,10 +7671,10 @@
         <v/>
       </c>
       <c r="L118" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M118" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SOCHNAYADOLINA-950-UNK-007. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N118">
         <v>500</v>
@@ -7689,16 +7689,16 @@
         <v>1</v>
       </c>
       <c r="R118">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S118" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T118" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U118" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="119">
@@ -7733,10 +7733,10 @@
         <v/>
       </c>
       <c r="L119" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M119" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SOCHNAYADOLINA-950-UNK-008. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N119">
         <v>500</v>
@@ -7751,16 +7751,16 @@
         <v>1</v>
       </c>
       <c r="R119">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S119" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T119" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U119" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="120">
@@ -7919,10 +7919,10 @@
         <v/>
       </c>
       <c r="L122" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M122" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SADYPRIDONYA-200-UNK-005. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N122">
         <v>1024</v>
@@ -7937,16 +7937,16 @@
         <v>1</v>
       </c>
       <c r="R122">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S122" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T122" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U122" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="123">
@@ -8229,10 +8229,10 @@
         <v/>
       </c>
       <c r="L127" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M127" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-MOI-200-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N127">
         <v>800</v>
@@ -8247,16 +8247,16 @@
         <v>1</v>
       </c>
       <c r="R127">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S127" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T127" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U127" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="128">
@@ -8291,10 +8291,10 @@
         <v/>
       </c>
       <c r="L128" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M128" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-MOI-200-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N128">
         <v>500</v>
@@ -8309,16 +8309,16 @@
         <v>1</v>
       </c>
       <c r="R128">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S128" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T128" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U128" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="129">
@@ -8353,10 +8353,10 @@
         <v/>
       </c>
       <c r="L129" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M129" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DOBRYI-2000-UNK-004. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N129">
         <v>1254</v>
@@ -8371,16 +8371,16 @@
         <v>1</v>
       </c>
       <c r="R129">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S129" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T129" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U129" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="130">
@@ -8657,10 +8657,10 @@
         <v/>
       </c>
       <c r="L134" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M134" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-LYUBIMYI-950-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N134">
         <v>500</v>
@@ -8675,16 +8675,16 @@
         <v>1</v>
       </c>
       <c r="R134">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S134" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T134" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U134" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="135">
@@ -8719,10 +8719,10 @@
         <v/>
       </c>
       <c r="L135" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M135" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-LYUBIMYI-950-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N135">
         <v>1000</v>
@@ -8737,16 +8737,16 @@
         <v>1</v>
       </c>
       <c r="R135">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S135" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T135" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U135" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="136">
@@ -8781,10 +8781,10 @@
         <v/>
       </c>
       <c r="L136" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M136" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-LYUBIMYI-950-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N136">
         <v>500</v>
@@ -8799,16 +8799,16 @@
         <v>1</v>
       </c>
       <c r="R136">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S136" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T136" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U136" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="137">
@@ -8843,10 +8843,10 @@
         <v/>
       </c>
       <c r="L137" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M137" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-LYUBIMYI-950-UNK-004. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N137">
         <v>500</v>
@@ -8861,16 +8861,16 @@
         <v>1</v>
       </c>
       <c r="R137">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S137" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T137" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U137" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="138">
@@ -8905,10 +8905,10 @@
         <v/>
       </c>
       <c r="L138" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M138" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-MOI-950-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N138">
         <v>600</v>
@@ -8923,16 +8923,16 @@
         <v>1</v>
       </c>
       <c r="R138">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S138" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T138" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U138" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="139">
@@ -8967,10 +8967,10 @@
         <v/>
       </c>
       <c r="L139" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M139" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-MOI-950-UNK-004. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N139">
         <v>600</v>
@@ -8985,16 +8985,16 @@
         <v>1</v>
       </c>
       <c r="R139">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S139" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T139" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U139" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="140">
@@ -9029,10 +9029,10 @@
         <v/>
       </c>
       <c r="L140" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M140" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-MOI-950-UNK-005. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N140">
         <v>600</v>
@@ -9047,16 +9047,16 @@
         <v>1</v>
       </c>
       <c r="R140">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S140" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T140" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U140" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="141">
@@ -9091,10 +9091,10 @@
         <v/>
       </c>
       <c r="L141" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M141" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VIKO-200-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N141">
         <v>500</v>
@@ -9109,16 +9109,16 @@
         <v>1</v>
       </c>
       <c r="R141">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S141" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T141" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U141" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="142">
@@ -9153,10 +9153,10 @@
         <v/>
       </c>
       <c r="L142" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M142" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VIKO-1000-UNK-011. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N142">
         <v>550</v>
@@ -9171,16 +9171,16 @@
         <v>1</v>
       </c>
       <c r="R142">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S142" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T142" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U142" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="143">
@@ -9215,10 +9215,10 @@
         <v/>
       </c>
       <c r="L143" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M143" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SANTAL-1000-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N143">
         <v>1024</v>
@@ -9233,16 +9233,16 @@
         <v>1</v>
       </c>
       <c r="R143">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S143" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T143" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U143" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="144">
@@ -9339,10 +9339,10 @@
         <v/>
       </c>
       <c r="L145" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M145" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SADYPRIDONYA-200-UNK-006. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N145">
         <v>1024</v>
@@ -9357,16 +9357,16 @@
         <v>1</v>
       </c>
       <c r="R145">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S145" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T145" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U145" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="146">
@@ -9401,10 +9401,10 @@
         <v/>
       </c>
       <c r="L146" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M146" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SOCHNAYADOLINA-1930-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N146">
         <v>600</v>
@@ -9419,16 +9419,16 @@
         <v>1</v>
       </c>
       <c r="R146">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S146" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T146" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U146" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="147">
@@ -9463,10 +9463,10 @@
         <v/>
       </c>
       <c r="L147" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M147" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SOCHNAYADOLINA-1930-UNK-004. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N147">
         <v>500</v>
@@ -9481,16 +9481,16 @@
         <v>1</v>
       </c>
       <c r="R147">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S147" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T147" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U147" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="148">
@@ -9649,10 +9649,10 @@
         <v/>
       </c>
       <c r="L150" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M150" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-MOI-200-UNK-004. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N150">
         <v>1000</v>
@@ -9667,16 +9667,16 @@
         <v>1</v>
       </c>
       <c r="R150">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S150" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T150" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U150" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="151">
@@ -9773,10 +9773,10 @@
         <v/>
       </c>
       <c r="L152" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M152" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DOBRYI-200-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N152">
         <v>1254</v>
@@ -9791,16 +9791,16 @@
         <v>1</v>
       </c>
       <c r="R152">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S152" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T152" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U152" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="153">
@@ -9835,10 +9835,10 @@
         <v/>
       </c>
       <c r="L153" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M153" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DOBRYI-200-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N153">
         <v>1024</v>
@@ -9853,16 +9853,16 @@
         <v>1</v>
       </c>
       <c r="R153">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S153" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T153" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U153" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="154">
@@ -10024,10 +10024,10 @@
         <v/>
       </c>
       <c r="L156" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M156" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-BAZIL-290-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N156">
         <v>500</v>
@@ -10042,16 +10042,16 @@
         <v>1</v>
       </c>
       <c r="R156">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S156" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice_drink</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice_drink</v>
       </c>
       <c r="T156" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U156" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="157">
@@ -10086,10 +10086,10 @@
         <v/>
       </c>
       <c r="L157" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M157" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SIS-1600-UNK-008. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N157">
         <v>1024</v>
@@ -10104,16 +10104,16 @@
         <v>1</v>
       </c>
       <c r="R157">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S157" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T157" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U157" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="158">
@@ -10148,10 +10148,10 @@
         <v/>
       </c>
       <c r="L158" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M158" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VIKO-1000-UNK-012. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N158">
         <v>500</v>
@@ -10166,16 +10166,16 @@
         <v>1</v>
       </c>
       <c r="R158">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S158" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T158" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U158" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="159">
@@ -10210,10 +10210,10 @@
         <v/>
       </c>
       <c r="L159" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M159" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-LYUBIMYI-200-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N159">
         <v>1024</v>
@@ -10228,16 +10228,16 @@
         <v>1</v>
       </c>
       <c r="R159">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S159" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T159" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U159" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="160">
@@ -10272,10 +10272,10 @@
         <v/>
       </c>
       <c r="L160" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M160" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-LYUBIMYI-950-UNK-005. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N160">
         <v>1000</v>
@@ -10290,16 +10290,16 @@
         <v>1</v>
       </c>
       <c r="R160">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S160" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T160" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U160" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="161">
@@ -10334,10 +10334,10 @@
         <v/>
       </c>
       <c r="L161" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M161" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-LYUBIMYI-1930-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N161">
         <v>600</v>
@@ -10352,16 +10352,16 @@
         <v>1</v>
       </c>
       <c r="R161">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S161" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T161" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U161" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="162">
@@ -10396,10 +10396,10 @@
         <v/>
       </c>
       <c r="L162" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M162" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-MOI-950-UNK-006. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N162">
         <v>600</v>
@@ -10414,16 +10414,16 @@
         <v>1</v>
       </c>
       <c r="R162">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S162" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T162" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U162" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="163">
@@ -10458,10 +10458,10 @@
         <v/>
       </c>
       <c r="L163" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M163" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-MOI-1930-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N163">
         <v>650</v>
@@ -10476,16 +10476,16 @@
         <v>1</v>
       </c>
       <c r="R163">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S163" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T163" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U163" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="164">
@@ -10520,10 +10520,10 @@
         <v/>
       </c>
       <c r="L164" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M164" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-MOI-1930-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N164">
         <v>650</v>
@@ -10538,16 +10538,16 @@
         <v>1</v>
       </c>
       <c r="R164">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S164" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T164" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U164" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="165">
@@ -10706,10 +10706,10 @@
         <v/>
       </c>
       <c r="L167" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M167" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-J7-970-UNK-006. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N167">
         <v>1024</v>
@@ -10724,16 +10724,16 @@
         <v>1</v>
       </c>
       <c r="R167">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S167" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T167" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U167" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="168">
@@ -10768,10 +10768,10 @@
         <v/>
       </c>
       <c r="L168" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M168" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VIKO-200-UNK-004. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N168">
         <v>500</v>
@@ -10786,16 +10786,16 @@
         <v>1</v>
       </c>
       <c r="R168">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S168" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T168" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U168" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="169">
@@ -10830,10 +10830,10 @@
         <v/>
       </c>
       <c r="L169" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M169" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VIKO-200-UNK-005. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N169">
         <v>680</v>
@@ -10848,16 +10848,16 @@
         <v>1</v>
       </c>
       <c r="R169">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S169" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T169" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U169" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="170">
@@ -10892,10 +10892,10 @@
         <v/>
       </c>
       <c r="L170" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M170" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SADYPRIDONYA-200-UNK-007. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N170">
         <v>1000</v>
@@ -10910,16 +10910,16 @@
         <v>1</v>
       </c>
       <c r="R170">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S170" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T170" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U170" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="171">
@@ -10954,10 +10954,10 @@
         <v/>
       </c>
       <c r="L171" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M171" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SADYPRIDONYA-1000-UNK-008. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N171">
         <v>1024</v>
@@ -10972,16 +10972,16 @@
         <v>1</v>
       </c>
       <c r="R171">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S171" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|marked_sugar_free|category_juice_slug|product_type_juice</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|marked_sugar_free|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T171" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U171" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="172">
@@ -11016,10 +11016,10 @@
         <v/>
       </c>
       <c r="L172" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M172" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SADYPRIDONYA-1000-UNK-009. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N172">
         <v>1024</v>
@@ -11034,16 +11034,16 @@
         <v>1</v>
       </c>
       <c r="R172">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S172" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|marked_sugar_free|category_juice_slug|product_type_juice|has_pulp</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|marked_sugar_free|category_juice_slug|product_type_juice|has_pulp</v>
       </c>
       <c r="T172" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U172" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="173">
@@ -11264,10 +11264,10 @@
         <v/>
       </c>
       <c r="L176" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M176" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SIS-1600-UNK-009. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N176">
         <v>1024</v>
@@ -11282,16 +11282,16 @@
         <v>1</v>
       </c>
       <c r="R176">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S176" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T176" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U176" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="177">
@@ -11326,10 +11326,10 @@
         <v/>
       </c>
       <c r="L177" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M177" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SOCHNAYADOLINA-200-UNK-005. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N177">
         <v>650</v>
@@ -11344,16 +11344,16 @@
         <v>1</v>
       </c>
       <c r="R177">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S177" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T177" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U177" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="178">
@@ -11388,10 +11388,10 @@
         <v/>
       </c>
       <c r="L178" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M178" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VINUT-330-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N178">
         <v>600</v>
@@ -11406,16 +11406,16 @@
         <v>1</v>
       </c>
       <c r="R178">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S178" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice_drink</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice_drink</v>
       </c>
       <c r="T178" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U178" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="179">
@@ -11636,10 +11636,10 @@
         <v/>
       </c>
       <c r="L182" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M182" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-VIKO-1000-UNK-013. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N182">
         <v>1000</v>
@@ -11654,16 +11654,16 @@
         <v>1</v>
       </c>
       <c r="R182">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S182" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T182" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U182" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="183">
@@ -11822,10 +11822,10 @@
         <v/>
       </c>
       <c r="L185" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M185" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DOBRYI-200-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N185">
         <v>1024</v>
@@ -11840,16 +11840,16 @@
         <v>1</v>
       </c>
       <c r="R185">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S185" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T185" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U185" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="186">
@@ -11949,10 +11949,10 @@
         <v/>
       </c>
       <c r="L187" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M187" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-FRUTONYANYA-200-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N187">
         <v>1024</v>
@@ -11967,16 +11967,16 @@
         <v>1</v>
       </c>
       <c r="R187">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S187" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line|clarified</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line|clarified</v>
       </c>
       <c r="T187" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U187" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="188">
@@ -12011,10 +12011,10 @@
         <v/>
       </c>
       <c r="L188" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M188" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-FRUTONYANYA-200-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N188">
         <v>900</v>
@@ -12029,16 +12029,16 @@
         <v>1</v>
       </c>
       <c r="R188">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S188" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line</v>
       </c>
       <c r="T188" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U188" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="189">
@@ -12073,10 +12073,10 @@
         <v/>
       </c>
       <c r="L189" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M189" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-FRUTONYANYA-200-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N189">
         <v>600</v>
@@ -12091,16 +12091,16 @@
         <v>1</v>
       </c>
       <c r="R189">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S189" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line|has_pulp</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line|has_pulp</v>
       </c>
       <c r="T189" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U189" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="190">
@@ -12135,10 +12135,10 @@
         <v/>
       </c>
       <c r="L190" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M190" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-FRUTONYANYA-200-UNK-004. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N190">
         <v>900</v>
@@ -12153,16 +12153,16 @@
         <v>1</v>
       </c>
       <c r="R190">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S190" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line|clarified</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line|clarified</v>
       </c>
       <c r="T190" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U190" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="191">
@@ -12197,10 +12197,10 @@
         <v/>
       </c>
       <c r="L191" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M191" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-FRUTONYANYA-200-UNK-005. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N191">
         <v>500</v>
@@ -12215,16 +12215,16 @@
         <v>1</v>
       </c>
       <c r="R191">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S191" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line</v>
       </c>
       <c r="T191" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U191" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="192">
@@ -12259,10 +12259,10 @@
         <v/>
       </c>
       <c r="L192" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M192" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-FRUTONYANYA-200-UNK-006. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N192">
         <v>500</v>
@@ -12277,16 +12277,16 @@
         <v>1</v>
       </c>
       <c r="R192">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S192" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line|has_pulp</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line|has_pulp</v>
       </c>
       <c r="T192" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U192" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="193">
@@ -12383,10 +12383,10 @@
         <v/>
       </c>
       <c r="L194" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M194" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-FRUTONYANYA-200-UNK-007. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N194">
         <v>900</v>
@@ -12401,16 +12401,16 @@
         <v>1</v>
       </c>
       <c r="R194">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S194" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line|has_pulp</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line|has_pulp</v>
       </c>
       <c r="T194" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U194" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="195">
@@ -12445,10 +12445,10 @@
         <v/>
       </c>
       <c r="L195" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M195" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DARYKUBANI-200-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N195">
         <v>650</v>
@@ -12463,16 +12463,16 @@
         <v>1</v>
       </c>
       <c r="R195">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S195" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line</v>
       </c>
       <c r="T195" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U195" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="196">
@@ -12631,10 +12631,10 @@
         <v/>
       </c>
       <c r="L198" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M198" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-FRUTONYANYA-500-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N198">
         <v>500</v>
@@ -12649,16 +12649,16 @@
         <v>1</v>
       </c>
       <c r="R198">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S198" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line</v>
       </c>
       <c r="T198" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U198" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="199">
@@ -12693,10 +12693,10 @@
         <v/>
       </c>
       <c r="L199" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M199" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-FRUTONYANYA-200-UNK-008. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N199">
         <v>909</v>
@@ -12711,16 +12711,16 @@
         <v>1</v>
       </c>
       <c r="R199">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S199" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line|has_pulp</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line|has_pulp</v>
       </c>
       <c r="T199" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U199" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="200">
@@ -12820,7 +12820,7 @@
         <v>needs_review</v>
       </c>
       <c r="M201" t="str">
-        <v>Авто: new_product, нужна ручная проверка (volume_missing)</v>
+        <v>Авто: new_product, нужна ручная проверка (volume_missing, package_missing, package_undetermined)</v>
       </c>
       <c r="N201">
         <v>650</v>
@@ -12838,10 +12838,10 @@
         <v>0.58</v>
       </c>
       <c r="S201" t="str">
-        <v>brand_parsed|name_present|flavor_present|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line</v>
+        <v>brand_parsed|name_present|flavor_present|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line</v>
       </c>
       <c r="T201" t="str">
-        <v>volume_missing</v>
+        <v>volume_missing|package_missing|package_undetermined</v>
       </c>
       <c r="U201" t="str">
         <v>needs_review_new_incomplete</v>
@@ -12941,10 +12941,10 @@
         <v/>
       </c>
       <c r="L203" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M203" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DARYKUBANI-200-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N203">
         <v>900</v>
@@ -12959,16 +12959,16 @@
         <v>1</v>
       </c>
       <c r="R203">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S203" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
       </c>
       <c r="T203" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U203" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="204">
@@ -13065,10 +13065,10 @@
         <v/>
       </c>
       <c r="L205" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M205" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-AGUSHA-200-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N205">
         <v>500</v>
@@ -13083,16 +13083,16 @@
         <v>1</v>
       </c>
       <c r="R205">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S205" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line|has_pulp</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line|has_pulp</v>
       </c>
       <c r="T205" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U205" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="206">
@@ -13189,10 +13189,10 @@
         <v/>
       </c>
       <c r="L207" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M207" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-FRUTONYANYA-200-UNK-010. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N207">
         <v>500</v>
@@ -13207,16 +13207,16 @@
         <v>1</v>
       </c>
       <c r="R207">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S207" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_mors|kids_line</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_mors|kids_line</v>
       </c>
       <c r="T207" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U207" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="208">
@@ -13251,10 +13251,10 @@
         <v/>
       </c>
       <c r="L208" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M208" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-FRUTONYANYA-200-UNK-011. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N208">
         <v>500</v>
@@ -13269,16 +13269,16 @@
         <v>1</v>
       </c>
       <c r="R208">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S208" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line|clarified</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line|clarified</v>
       </c>
       <c r="T208" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U208" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="209">
@@ -13313,10 +13313,10 @@
         <v/>
       </c>
       <c r="L209" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M209" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DARYKUBANI-200-UNK-005. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N209">
         <v>1024</v>
@@ -13331,16 +13331,16 @@
         <v>1</v>
       </c>
       <c r="R209">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S209" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line|clarified</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line|clarified</v>
       </c>
       <c r="T209" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U209" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="210">
@@ -13375,10 +13375,10 @@
         <v/>
       </c>
       <c r="L210" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M210" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-AGUSHA-200-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N210">
         <v>500</v>
@@ -13393,16 +13393,16 @@
         <v>1</v>
       </c>
       <c r="R210">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S210" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line|clarified</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line|clarified</v>
       </c>
       <c r="T210" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U210" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="211">
@@ -13437,10 +13437,10 @@
         <v/>
       </c>
       <c r="L211" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M211" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-AGUSHA-200-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N211">
         <v>1250</v>
@@ -13455,16 +13455,16 @@
         <v>1</v>
       </c>
       <c r="R211">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S211" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line|clarified</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line|clarified</v>
       </c>
       <c r="T211" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U211" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="212">
@@ -13499,10 +13499,10 @@
         <v/>
       </c>
       <c r="L212" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M212" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DARYKUBANI-200-UNK-006. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N212">
         <v>700</v>
@@ -13517,16 +13517,16 @@
         <v>1</v>
       </c>
       <c r="R212">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S212" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
       </c>
       <c r="T212" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U212" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="213">
@@ -13561,10 +13561,10 @@
         <v/>
       </c>
       <c r="L213" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M213" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-FRUTONYANYA-500-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N213">
         <v>1024</v>
@@ -13579,16 +13579,16 @@
         <v>1</v>
       </c>
       <c r="R213">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S213" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line|has_pulp</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line|has_pulp</v>
       </c>
       <c r="T213" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U213" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="214">
@@ -13623,10 +13623,10 @@
         <v/>
       </c>
       <c r="L214" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M214" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-FRUTONYANYA-500-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N214">
         <v>650</v>
@@ -13641,16 +13641,16 @@
         <v>1</v>
       </c>
       <c r="R214">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S214" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line|has_pulp</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line|has_pulp</v>
       </c>
       <c r="T214" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U214" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="215">
@@ -13685,10 +13685,10 @@
         <v/>
       </c>
       <c r="L215" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M215" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-MALENKOESCHASTE-200-UNK-001. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N215">
         <v>500</v>
@@ -13703,16 +13703,16 @@
         <v>1</v>
       </c>
       <c r="R215">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S215" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
       </c>
       <c r="T215" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U215" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="216">
@@ -13747,10 +13747,10 @@
         <v/>
       </c>
       <c r="L216" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M216" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DARYKUBANI-200-UNK-007. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N216">
         <v>1024</v>
@@ -13765,16 +13765,16 @@
         <v>1</v>
       </c>
       <c r="R216">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S216" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line|has_pulp</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line|has_pulp</v>
       </c>
       <c r="T216" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U216" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="217">
@@ -13809,10 +13809,10 @@
         <v/>
       </c>
       <c r="L217" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M217" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DARYKUBANI-200-UNK-008. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N217">
         <v>500</v>
@@ -13827,16 +13827,16 @@
         <v>1</v>
       </c>
       <c r="R217">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S217" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
       </c>
       <c r="T217" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U217" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="218">
@@ -13871,10 +13871,10 @@
         <v/>
       </c>
       <c r="L218" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M218" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-MALENKOESCHASTE-200-UNK-002. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N218">
         <v>550</v>
@@ -13889,16 +13889,16 @@
         <v>1</v>
       </c>
       <c r="R218">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S218" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
       </c>
       <c r="T218" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U218" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="219">
@@ -13933,10 +13933,10 @@
         <v/>
       </c>
       <c r="L219" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M219" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-MALENKOESCHASTE-200-UNK-003. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N219">
         <v>1024</v>
@@ -13951,16 +13951,16 @@
         <v>1</v>
       </c>
       <c r="R219">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S219" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
       </c>
       <c r="T219" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U219" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="220">
@@ -13998,7 +13998,7 @@
         <v>needs_review</v>
       </c>
       <c r="M220" t="str">
-        <v>Авто: new_product, нужна ручная проверка (volume_missing)</v>
+        <v>Авто: new_product, нужна ручная проверка (volume_missing, package_missing, package_undetermined)</v>
       </c>
       <c r="N220">
         <v>500</v>
@@ -14016,10 +14016,10 @@
         <v>0.58</v>
       </c>
       <c r="S220" t="str">
-        <v>brand_parsed|name_present|flavor_present|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line|clarified</v>
+        <v>brand_parsed|name_present|flavor_present|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line|clarified</v>
       </c>
       <c r="T220" t="str">
-        <v>volume_missing</v>
+        <v>volume_missing|package_missing|package_undetermined</v>
       </c>
       <c r="U220" t="str">
         <v>needs_review_new_incomplete</v>
@@ -14060,7 +14060,7 @@
         <v>needs_review</v>
       </c>
       <c r="M221" t="str">
-        <v>Авто: new_product, нужна ручная проверка (volume_missing)</v>
+        <v>Авто: new_product, нужна ручная проверка (volume_missing, package_missing, package_undetermined)</v>
       </c>
       <c r="N221">
         <v>500</v>
@@ -14078,10 +14078,10 @@
         <v>0.58</v>
       </c>
       <c r="S221" t="str">
-        <v>brand_parsed|name_present|flavor_present|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
+        <v>brand_parsed|name_present|flavor_present|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
       </c>
       <c r="T221" t="str">
-        <v>volume_missing</v>
+        <v>volume_missing|package_missing|package_undetermined</v>
       </c>
       <c r="U221" t="str">
         <v>needs_review_new_incomplete</v>
@@ -14119,10 +14119,10 @@
         <v/>
       </c>
       <c r="L222" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M222" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-MALENKOESCHASTE-200-UNK-004. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N222">
         <v>800</v>
@@ -14137,16 +14137,16 @@
         <v>1</v>
       </c>
       <c r="R222">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S222" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
       </c>
       <c r="T222" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U222" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="223">
@@ -14181,10 +14181,10 @@
         <v/>
       </c>
       <c r="L223" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M223" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-AGUSHA-200-UNK-004. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N223">
         <v>500</v>
@@ -14199,16 +14199,16 @@
         <v>1</v>
       </c>
       <c r="R223">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S223" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line|has_pulp</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line|has_pulp</v>
       </c>
       <c r="T223" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U223" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="224">
@@ -14243,10 +14243,10 @@
         <v/>
       </c>
       <c r="L224" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M224" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-AGUSHA-200-UNK-005. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N224">
         <v>500</v>
@@ -14261,16 +14261,16 @@
         <v>1</v>
       </c>
       <c r="R224">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S224" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line|clarified</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line|clarified</v>
       </c>
       <c r="T224" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U224" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="225">
@@ -14367,10 +14367,10 @@
         <v/>
       </c>
       <c r="L226" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M226" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-MALENKOESCHASTE-200-UNK-006. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N226">
         <v>600</v>
@@ -14385,16 +14385,16 @@
         <v>1</v>
       </c>
       <c r="R226">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S226" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
       </c>
       <c r="T226" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U226" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="227">
@@ -14429,10 +14429,10 @@
         <v/>
       </c>
       <c r="L227" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M227" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-AGUSHA-200-UNK-006. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N227">
         <v>500</v>
@@ -14447,16 +14447,16 @@
         <v>1</v>
       </c>
       <c r="R227">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S227" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line|has_pulp</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line|has_pulp</v>
       </c>
       <c r="T227" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U227" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="228">
@@ -14491,10 +14491,10 @@
         <v/>
       </c>
       <c r="L228" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M228" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-MALENKOESCHASTE-200-UNK-007. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N228">
         <v>1024</v>
@@ -14509,16 +14509,16 @@
         <v>1</v>
       </c>
       <c r="R228">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S228" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
       </c>
       <c r="T228" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U228" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="229">
@@ -14553,10 +14553,10 @@
         <v/>
       </c>
       <c r="L229" t="str">
-        <v>approved_new</v>
+        <v>needs_review</v>
       </c>
       <c r="M229" t="str">
-        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-AGUSHA-200-UNK-007. Товар ещё не создан — только кандидат.</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N229">
         <v>500</v>
@@ -14571,16 +14571,16 @@
         <v>1</v>
       </c>
       <c r="R229">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="S229" t="str">
-        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line|clarified</v>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line|clarified</v>
       </c>
       <c r="T229" t="str">
-        <v/>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U229" t="str">
-        <v>approved_new_clean_candidate</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="230">

</xml_diff>

<commit_message>
fix(catalog): do not exclude grape juice as wine in auto-review
Co-authored-by: sharipdaitmirzaev-hue <sharipdaitmirzaev-hue@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/imports/zelenoe-yabloko-juice/review-decisions.xlsx
+++ b/data/imports/zelenoe-yabloko-juice/review-decisions.xlsx
@@ -2487,10 +2487,10 @@
         <v/>
       </c>
       <c r="L34" t="str">
-        <v>rejected</v>
+        <v>approved_new</v>
       </c>
       <c r="M34" t="str">
-        <v>Авто: excluded-категория / не целевой напиток</v>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-IRIB-750-GLASS-008. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N34">
         <v>600</v>
@@ -2505,16 +2505,16 @@
         <v>1</v>
       </c>
       <c r="R34">
-        <v>0.85</v>
+        <v>0.78</v>
       </c>
       <c r="S34" t="str">
-        <v/>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T34" t="str">
-        <v>excluded_category</v>
+        <v/>
       </c>
       <c r="U34" t="str">
-        <v>rejected_excluded_category</v>
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="35">
@@ -2983,10 +2983,10 @@
         <v/>
       </c>
       <c r="L42" t="str">
-        <v>rejected</v>
+        <v>needs_review</v>
       </c>
       <c r="M42" t="str">
-        <v>Авто: excluded-категория / не целевой напиток</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N42">
         <v>550</v>
@@ -3001,16 +3001,16 @@
         <v>1</v>
       </c>
       <c r="R42">
-        <v>0.85</v>
+        <v>0.58</v>
       </c>
       <c r="S42" t="str">
-        <v/>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T42" t="str">
-        <v>excluded_category</v>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U42" t="str">
-        <v>rejected_excluded_category</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="43">
@@ -4474,10 +4474,10 @@
         <v/>
       </c>
       <c r="L66" t="str">
-        <v>rejected</v>
+        <v>needs_review</v>
       </c>
       <c r="M66" t="str">
-        <v>Авто: excluded-категория / не целевой напиток</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N66">
         <v>1024</v>
@@ -4492,16 +4492,16 @@
         <v>1</v>
       </c>
       <c r="R66">
-        <v>0.85</v>
+        <v>0.58</v>
       </c>
       <c r="S66" t="str">
-        <v/>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T66" t="str">
-        <v>excluded_category</v>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U66" t="str">
-        <v>rejected_excluded_category</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="67">
@@ -6251,10 +6251,10 @@
         <v/>
       </c>
       <c r="L95" t="str">
-        <v>rejected</v>
+        <v>needs_review</v>
       </c>
       <c r="M95" t="str">
-        <v>Авто: excluded-категория / не целевой напиток</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N95">
         <v>550</v>
@@ -6269,16 +6269,16 @@
         <v>1</v>
       </c>
       <c r="R95">
-        <v>0.85</v>
+        <v>0.58</v>
       </c>
       <c r="S95" t="str">
-        <v/>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T95" t="str">
-        <v>excluded_category</v>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U95" t="str">
-        <v>rejected_excluded_category</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="96">
@@ -8167,10 +8167,10 @@
         <v/>
       </c>
       <c r="L126" t="str">
-        <v>rejected</v>
+        <v>approved_new</v>
       </c>
       <c r="M126" t="str">
-        <v>Авто: excluded-категория / не целевой напиток</v>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-KIKUNI-750-GLASS-003. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N126">
         <v>1024</v>
@@ -8185,16 +8185,16 @@
         <v>1</v>
       </c>
       <c r="R126">
-        <v>0.85</v>
+        <v>0.78</v>
       </c>
       <c r="S126" t="str">
-        <v/>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T126" t="str">
-        <v>excluded_category</v>
+        <v/>
       </c>
       <c r="U126" t="str">
-        <v>rejected_excluded_category</v>
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="127">
@@ -9277,10 +9277,10 @@
         <v/>
       </c>
       <c r="L144" t="str">
-        <v>rejected</v>
+        <v>approved_new</v>
       </c>
       <c r="M144" t="str">
-        <v>Авто: excluded-категория / не целевой напиток</v>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-GUNIB-750-GLASS-004. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N144">
         <v>1024</v>
@@ -9295,16 +9295,16 @@
         <v>1</v>
       </c>
       <c r="R144">
-        <v>0.85</v>
+        <v>0.78</v>
       </c>
       <c r="S144" t="str">
-        <v/>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice</v>
       </c>
       <c r="T144" t="str">
-        <v>excluded_category</v>
+        <v/>
       </c>
       <c r="U144" t="str">
-        <v>rejected_excluded_category</v>
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="145">
@@ -10582,10 +10582,10 @@
         <v/>
       </c>
       <c r="L165" t="str">
-        <v>rejected</v>
+        <v>needs_review</v>
       </c>
       <c r="M165" t="str">
-        <v>Авто: excluded-категория / не целевой напиток</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N165">
         <v>500</v>
@@ -10600,16 +10600,16 @@
         <v>1</v>
       </c>
       <c r="R165">
-        <v>0.85</v>
+        <v>0.58</v>
       </c>
       <c r="S165" t="str">
-        <v/>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar</v>
       </c>
       <c r="T165" t="str">
-        <v>excluded_category</v>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U165" t="str">
-        <v>rejected_excluded_category</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="166">
@@ -12507,10 +12507,10 @@
         <v/>
       </c>
       <c r="L196" t="str">
-        <v>rejected</v>
+        <v>approved_new</v>
       </c>
       <c r="M196" t="str">
-        <v>Авто: excluded-категория / не целевой напиток</v>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-AGUSHA-300-PET-002. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N196">
         <v>650</v>
@@ -12525,16 +12525,16 @@
         <v>1</v>
       </c>
       <c r="R196">
-        <v>0.85</v>
+        <v>0.78</v>
       </c>
       <c r="S196" t="str">
-        <v/>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice_drink|kids_line</v>
       </c>
       <c r="T196" t="str">
-        <v>excluded_category</v>
+        <v/>
       </c>
       <c r="U196" t="str">
-        <v>rejected_excluded_category</v>
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="197">
@@ -12879,10 +12879,10 @@
         <v/>
       </c>
       <c r="L202" t="str">
-        <v>rejected</v>
+        <v>needs_review</v>
       </c>
       <c r="M202" t="str">
-        <v>Авто: excluded-категория / не целевой напиток</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N202">
         <v>1024</v>
@@ -12897,16 +12897,16 @@
         <v>1</v>
       </c>
       <c r="R202">
-        <v>0.85</v>
+        <v>0.58</v>
       </c>
       <c r="S202" t="str">
-        <v/>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_juice|kids_line|clarified</v>
       </c>
       <c r="T202" t="str">
-        <v>excluded_category</v>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U202" t="str">
-        <v>rejected_excluded_category</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="203">
@@ -14305,10 +14305,10 @@
         <v/>
       </c>
       <c r="L225" t="str">
-        <v>rejected</v>
+        <v>needs_review</v>
       </c>
       <c r="M225" t="str">
-        <v>Авто: excluded-категория / не целевой напиток</v>
+        <v>Авто: new_product, нужна ручная проверка (package_missing, package_undetermined)</v>
       </c>
       <c r="N225">
         <v>1024</v>
@@ -14323,16 +14323,16 @@
         <v>1</v>
       </c>
       <c r="R225">
-        <v>0.85</v>
+        <v>0.58</v>
       </c>
       <c r="S225" t="str">
-        <v/>
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|category_juice_slug|product_type_nectar|kids_line</v>
       </c>
       <c r="T225" t="str">
-        <v>excluded_category</v>
+        <v>package_missing|package_undetermined</v>
       </c>
       <c r="U225" t="str">
-        <v>rejected_excluded_category</v>
+        <v>needs_review_new_incomplete</v>
       </c>
     </row>
     <row r="226">

</xml_diff>